<commit_message>
update on biomass potential
</commit_message>
<xml_diff>
--- a/data/carriers_data/MPW/MPW_availability.xlsx
+++ b/data/carriers_data/MPW/MPW_availability.xlsx
@@ -1,26 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\AdOpT-NET0_my\data\carriers_data\MPW\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAA2E6C6-EAF2-4BA0-AD89-B1BFB5E20FD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6148F1C4-93DA-4D41-A73E-C82B844E8137}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="note" sheetId="2" r:id="rId1"/>
     <sheet name="PP" sheetId="1" r:id="rId2"/>
     <sheet name="DA" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -396,13 +407,16 @@
         <v>392</v>
       </c>
       <c r="C2">
-        <v>392</v>
+        <f>$B2*C$4/$B$4</f>
+        <v>555.69230769230774</v>
       </c>
       <c r="D2">
-        <v>392</v>
+        <f t="shared" ref="D2:E3" si="0">$B2*D$4/$B$4</f>
+        <v>430.76923076923077</v>
       </c>
       <c r="E2">
-        <v>392</v>
+        <f t="shared" si="0"/>
+        <v>430.76923076923077</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -413,13 +427,16 @@
         <v>759</v>
       </c>
       <c r="C3">
-        <v>759</v>
+        <f>$B3*C$4/$B$4</f>
+        <v>1075.9450549450548</v>
       </c>
       <c r="D3">
-        <v>759</v>
+        <f t="shared" si="0"/>
+        <v>834.06593406593402</v>
       </c>
       <c r="E3">
-        <v>759</v>
+        <f t="shared" si="0"/>
+        <v>834.06593406593402</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>